<commit_message>
Update internship project files
</commit_message>
<xml_diff>
--- a/timesheet/manoj_timesheet.xlsx
+++ b/timesheet/manoj_timesheet.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="24">
   <si>
     <t>Date</t>
   </si>
@@ -78,16 +78,19 @@
     <t>one feature in Git, the git keep</t>
   </si>
   <si>
-    <t xml:space="preserve">Create the Maven analytics KPI summary. </t>
-  </si>
-  <si>
-    <t>Gemini for Excel formulae</t>
-  </si>
-  <si>
-    <t>used to get formulae to create the KPI summary.</t>
-  </si>
-  <si>
-    <t>few excel formulae, how they work, and how it can be used.</t>
+    <t>Create the Maven analytics KPI summary. Create  a kpi tree for namma metro</t>
+  </si>
+  <si>
+    <t>Gemini for Excel formulae, chatagpt for knowledge</t>
+  </si>
+  <si>
+    <t>used to get formulae to create the KPI summary, to learn about kpi trees</t>
+  </si>
+  <si>
+    <t>what are kpi trees</t>
+  </si>
+  <si>
+    <t xml:space="preserve">kpi_tree.md </t>
   </si>
 </sst>
 </file>
@@ -132,7 +135,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
@@ -146,6 +149,10 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -579,23 +586,32 @@
         <v>18</v>
       </c>
     </row>
-    <row r="7" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B7" s="1">
         <v>46315</v>
       </c>
       <c r="C7">
         <v>4</v>
       </c>
-      <c r="G7" t="s">
+      <c r="D7" s="6">
+        <v>0.77083333333333337</v>
+      </c>
+      <c r="E7" s="6">
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="F7">
+        <v>1.5</v>
+      </c>
+      <c r="G7" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="H7" t="s">
+      <c r="H7" s="7" t="s">
         <v>20</v>
       </c>
       <c r="I7" t="s">
-        <v>11</v>
-      </c>
-      <c r="J7" t="s">
+        <v>23</v>
+      </c>
+      <c r="J7" s="7" t="s">
         <v>21</v>
       </c>
       <c r="K7" t="s">

</xml_diff>

<commit_message>
Update internship project files(Day 4)
</commit_message>
<xml_diff>
--- a/timesheet/manoj_timesheet.xlsx
+++ b/timesheet/manoj_timesheet.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="28">
   <si>
     <t>Date</t>
   </si>
@@ -90,7 +90,19 @@
     <t>what are kpi trees</t>
   </si>
   <si>
-    <t xml:space="preserve">kpi_tree.md </t>
+    <t>https://github.com/manuhatescoding/mvj-internship-data-analytics/commit/1529c49ceaf36bfb142e524042aec15358fcd12c</t>
+  </si>
+  <si>
+    <t>complete project 1(Coffee shop analysis).</t>
+  </si>
+  <si>
+    <t>chatgpt</t>
+  </si>
+  <si>
+    <t>used to get and understand formulae(sumifs, xlookup)</t>
+  </si>
+  <si>
+    <t>none</t>
   </si>
 </sst>
 </file>
@@ -135,7 +147,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
@@ -154,6 +166,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -608,7 +621,7 @@
       <c r="H7" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="I7" t="s">
+      <c r="I7" s="8" t="s">
         <v>23</v>
       </c>
       <c r="J7" s="7" t="s">
@@ -625,6 +638,24 @@
       <c r="B8" s="1">
         <v>46316</v>
       </c>
+      <c r="C8">
+        <v>5</v>
+      </c>
+      <c r="D8" s="6">
+        <v>0.69444444444444453</v>
+      </c>
+      <c r="G8" t="s">
+        <v>24</v>
+      </c>
+      <c r="H8" t="s">
+        <v>25</v>
+      </c>
+      <c r="J8" t="s">
+        <v>26</v>
+      </c>
+      <c r="K8" t="s">
+        <v>27</v>
+      </c>
     </row>
     <row r="9" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B9" s="1">
@@ -639,6 +670,7 @@
   </sheetData>
   <hyperlinks>
     <hyperlink ref="I6" r:id="rId1"/>
+    <hyperlink ref="I7" r:id="rId2"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Update internship project files(day 7 tasks)
</commit_message>
<xml_diff>
--- a/timesheet/manoj_timesheet.xlsx
+++ b/timesheet/manoj_timesheet.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="38">
   <si>
     <t>Date</t>
   </si>
@@ -78,9 +78,6 @@
     <t>one feature in Git, the git keep</t>
   </si>
   <si>
-    <t>Create the Maven analytics KPI summary. Create  a kpi tree for namma metro</t>
-  </si>
-  <si>
     <t>Gemini for Excel formulae, chatagpt for knowledge</t>
   </si>
   <si>
@@ -118,6 +115,24 @@
   </si>
   <si>
     <t>https://github.com/manuhatescoding/mvj-internship-data-analytics/commit/8c3b3576a661f0c1c271f88ae1c6608c8b6c26dc</t>
+  </si>
+  <si>
+    <t>Create the Maven analytics KPI summary. Create  a kpi tree for namma metro, learnt the different types of analyses</t>
+  </si>
+  <si>
+    <t>complete day 6 tasks. JOINS  and CASE-based segments</t>
+  </si>
+  <si>
+    <t>https://github.com/manuhatescoding/mvj-internship-data-analytics/commit/030fbd06953f3d63443fbf8bc374d611f1872a5b</t>
+  </si>
+  <si>
+    <t>few git commands</t>
+  </si>
+  <si>
+    <t>complete day 7 tasks</t>
+  </si>
+  <si>
+    <t>multiple sql statements, joins, case funtions</t>
   </si>
 </sst>
 </file>
@@ -463,13 +478,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B3:L10"/>
+  <dimension ref="B3:L11"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="12.109375" customWidth="1"/>
     <col min="7" max="7" width="42" customWidth="1"/>
     <col min="8" max="8" width="23.21875" customWidth="1"/>
-    <col min="9" max="9" width="17.6640625" customWidth="1"/>
+    <col min="9" max="9" width="44" customWidth="1"/>
     <col min="10" max="10" width="44.44140625" customWidth="1"/>
     <col min="12" max="12" width="18" customWidth="1"/>
   </cols>
@@ -614,7 +629,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="7" spans="2:12" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B7" s="1">
         <v>46315</v>
       </c>
@@ -625,28 +640,28 @@
         <v>0.77083333333333337</v>
       </c>
       <c r="E7" s="6">
-        <v>0.83333333333333337</v>
+        <v>0.89583333333333337</v>
       </c>
       <c r="F7">
-        <v>1.5</v>
+        <v>3</v>
       </c>
       <c r="G7" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="H7" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="H7" s="7" t="s">
+      <c r="I7" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="J7" s="7" t="s">
         <v>20</v>
-      </c>
-      <c r="I7" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="J7" s="7" t="s">
-        <v>21</v>
       </c>
       <c r="K7" t="s">
         <v>17</v>
       </c>
       <c r="L7" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="8" spans="2:12" x14ac:dyDescent="0.3">
@@ -666,19 +681,19 @@
         <v>1.5</v>
       </c>
       <c r="G8" t="s">
+        <v>23</v>
+      </c>
+      <c r="H8" t="s">
         <v>24</v>
       </c>
-      <c r="H8" t="s">
+      <c r="I8" t="s">
+        <v>27</v>
+      </c>
+      <c r="J8" t="s">
         <v>25</v>
       </c>
-      <c r="I8" t="s">
-        <v>28</v>
-      </c>
-      <c r="J8" t="s">
+      <c r="K8" t="s">
         <v>26</v>
-      </c>
-      <c r="K8" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="9" spans="2:12" x14ac:dyDescent="0.3">
@@ -691,28 +706,96 @@
       <c r="D9" s="6">
         <v>0.70833333333333337</v>
       </c>
+      <c r="E9" s="6">
+        <v>0.8125</v>
+      </c>
+      <c r="F9">
+        <v>2.5</v>
+      </c>
       <c r="G9" t="s">
+        <v>28</v>
+      </c>
+      <c r="H9" t="s">
+        <v>24</v>
+      </c>
+      <c r="I9" t="s">
+        <v>31</v>
+      </c>
+      <c r="J9" t="s">
         <v>29</v>
       </c>
-      <c r="H9" t="s">
-        <v>25</v>
-      </c>
-      <c r="I9" t="s">
-        <v>32</v>
-      </c>
-      <c r="J9" t="s">
+      <c r="K9" t="s">
+        <v>26</v>
+      </c>
+      <c r="L9" t="s">
         <v>30</v>
       </c>
-      <c r="K9" t="s">
-        <v>27</v>
-      </c>
-      <c r="L9" t="s">
-        <v>31</v>
-      </c>
     </row>
-    <row r="10" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:12" ht="57.6" x14ac:dyDescent="0.3">
       <c r="B10" s="1">
         <v>46318</v>
+      </c>
+      <c r="C10">
+        <v>7</v>
+      </c>
+      <c r="D10" s="6">
+        <v>0.35416666666666669</v>
+      </c>
+      <c r="E10" s="6">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="F10">
+        <v>1.5</v>
+      </c>
+      <c r="G10" t="s">
+        <v>33</v>
+      </c>
+      <c r="H10" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="I10" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="J10" t="s">
+        <v>29</v>
+      </c>
+      <c r="K10" t="s">
+        <v>26</v>
+      </c>
+      <c r="L10" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="11" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B11" s="1">
+        <v>46318</v>
+      </c>
+      <c r="C11">
+        <v>7</v>
+      </c>
+      <c r="D11" s="6">
+        <v>0.72916666666666663</v>
+      </c>
+      <c r="E11" s="6">
+        <v>0.79166666666666663</v>
+      </c>
+      <c r="F11">
+        <v>2</v>
+      </c>
+      <c r="G11" t="s">
+        <v>36</v>
+      </c>
+      <c r="H11" t="s">
+        <v>24</v>
+      </c>
+      <c r="J11" t="s">
+        <v>29</v>
+      </c>
+      <c r="K11" t="s">
+        <v>26</v>
+      </c>
+      <c r="L11" t="s">
+        <v>37</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update internship project files(Day 8 tasks)
</commit_message>
<xml_diff>
--- a/timesheet/manoj_timesheet.xlsx
+++ b/timesheet/manoj_timesheet.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="45">
   <si>
     <t>Date</t>
   </si>
@@ -133,13 +133,38 @@
   </si>
   <si>
     <t>multiple sql statements, joins, case funtions</t>
+  </si>
+  <si>
+    <t>learn Descriptive, diagnostic,
+predictive, prescriptive
+analytics, Goal Seek, Data Tables,
+Scenario Manager, Forecast
+Sheet</t>
+  </si>
+  <si>
+    <t>https://github.com/manuhatescoding/mvj-internship-data-analytics/commit/d01c710aa01f51f897cfada034737ac6051ec1f0</t>
+  </si>
+  <si>
+    <t>used for learning various types of analyses, few excel functions</t>
+  </si>
+  <si>
+    <t>types of analyses</t>
+  </si>
+  <si>
+    <t>finish the project 1, kpi summary, understand each kpis, finding recommendations</t>
+  </si>
+  <si>
+    <t xml:space="preserve">used to get an idea of the kpis, </t>
+  </si>
+  <si>
+    <t>various kpis and their meanings</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -151,6 +176,14 @@
       <u/>
       <sz val="11"/>
       <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -177,7 +210,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
@@ -197,6 +230,10 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -478,7 +515,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B3:L11"/>
+  <dimension ref="B3:L13"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="12.109375" customWidth="1"/>
@@ -489,38 +526,38 @@
     <col min="12" max="12" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B3" t="s">
+    <row r="3" spans="2:12" s="10" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B3" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="E3" t="s">
+      <c r="E3" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="F3" t="s">
+      <c r="F3" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="G3" t="s">
+      <c r="G3" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="H3" t="s">
+      <c r="H3" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="I3" t="s">
+      <c r="I3" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="J3" t="s">
+      <c r="J3" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="K3" t="s">
+      <c r="K3" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="L3" t="s">
+      <c r="L3" s="10" t="s">
         <v>10</v>
       </c>
     </row>
@@ -796,12 +833,80 @@
       </c>
       <c r="L11" t="s">
         <v>37</v>
+      </c>
+    </row>
+    <row r="12" spans="2:12" ht="72" x14ac:dyDescent="0.3">
+      <c r="B12" s="1">
+        <v>46318</v>
+      </c>
+      <c r="C12">
+        <v>7</v>
+      </c>
+      <c r="D12" s="6">
+        <v>0.875</v>
+      </c>
+      <c r="E12" s="6">
+        <v>0.91666666666666663</v>
+      </c>
+      <c r="F12">
+        <v>1</v>
+      </c>
+      <c r="G12" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="H12" t="s">
+        <v>24</v>
+      </c>
+      <c r="I12" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="J12" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="K12" t="s">
+        <v>17</v>
+      </c>
+      <c r="L12" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="13" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B13" s="1">
+        <v>46319</v>
+      </c>
+      <c r="C13">
+        <v>8</v>
+      </c>
+      <c r="D13" s="6">
+        <v>0.35416666666666669</v>
+      </c>
+      <c r="E13" s="6">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="F13">
+        <v>1.5</v>
+      </c>
+      <c r="G13" t="s">
+        <v>42</v>
+      </c>
+      <c r="H13" t="s">
+        <v>24</v>
+      </c>
+      <c r="J13" t="s">
+        <v>43</v>
+      </c>
+      <c r="K13" t="s">
+        <v>17</v>
+      </c>
+      <c r="L13" t="s">
+        <v>44</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="I6" r:id="rId1"/>
     <hyperlink ref="I7" r:id="rId2"/>
+    <hyperlink ref="I12" r:id="rId3"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Upload day 10 tasks
</commit_message>
<xml_diff>
--- a/timesheet/manoj_timesheet.xlsx
+++ b/timesheet/manoj_timesheet.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="56">
   <si>
     <t>Date</t>
   </si>
@@ -151,13 +151,46 @@
     <t>types of analyses</t>
   </si>
   <si>
-    <t>finish the project 1, kpi summary, understand each kpis, finding recommendations</t>
-  </si>
-  <si>
-    <t xml:space="preserve">used to get an idea of the kpis, </t>
-  </si>
-  <si>
     <t>various kpis and their meanings</t>
+  </si>
+  <si>
+    <t>https://github.com/manuhatescoding/mvj-internship-data-analytics/commit/dfe7b2d32dee13feb169cd8175b31a67b2befff9</t>
+  </si>
+  <si>
+    <t>used to get an idea of the kpis, its types and its meanings.</t>
+  </si>
+  <si>
+    <t>SQLBolt</t>
+  </si>
+  <si>
+    <t>finish SQLB lessons 1-8, finish Kaggle Python lessons 1-3 and exercises</t>
+  </si>
+  <si>
+    <t>sql basics, python functions advanced</t>
+  </si>
+  <si>
+    <t>finish the project 1(day 8 tasks), kpi summary, understand each kpis, finding recommendations</t>
+  </si>
+  <si>
+    <t>finish SQLB lessons 9-11, KG-PY lessons 2-4</t>
+  </si>
+  <si>
+    <t>SQLBolt, Kaggle</t>
+  </si>
+  <si>
+    <t>multiple SQL functions, Python functions and arguments</t>
+  </si>
+  <si>
+    <t>finish Day 19 tasks(recreate project 1 using pandas)</t>
+  </si>
+  <si>
+    <t>Google Colab, chatgpt</t>
+  </si>
+  <si>
+    <t>used to get pandas code</t>
+  </si>
+  <si>
+    <t>various functions used in pandas</t>
   </si>
 </sst>
 </file>
@@ -515,7 +548,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B3:L13"/>
+  <dimension ref="B3:L16"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="12.109375" customWidth="1"/>
@@ -887,19 +920,118 @@
         <v>1.5</v>
       </c>
       <c r="G13" t="s">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="H13" t="s">
         <v>24</v>
       </c>
+      <c r="I13" s="8" t="s">
+        <v>43</v>
+      </c>
       <c r="J13" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="K13" t="s">
         <v>17</v>
       </c>
       <c r="L13" t="s">
-        <v>44</v>
+        <v>42</v>
+      </c>
+    </row>
+    <row r="14" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B14" s="1">
+        <v>46319</v>
+      </c>
+      <c r="C14">
+        <v>8</v>
+      </c>
+      <c r="D14" s="6">
+        <v>0.58333333333333337</v>
+      </c>
+      <c r="E14" s="6">
+        <v>0.70833333333333337</v>
+      </c>
+      <c r="F14">
+        <v>3</v>
+      </c>
+      <c r="G14" t="s">
+        <v>46</v>
+      </c>
+      <c r="H14" t="s">
+        <v>45</v>
+      </c>
+      <c r="J14" t="s">
+        <v>11</v>
+      </c>
+      <c r="K14" t="s">
+        <v>26</v>
+      </c>
+      <c r="L14" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="15" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B15" s="1">
+        <v>46320</v>
+      </c>
+      <c r="C15">
+        <v>9</v>
+      </c>
+      <c r="D15" s="6">
+        <v>0.375</v>
+      </c>
+      <c r="E15" s="6">
+        <v>0.5</v>
+      </c>
+      <c r="F15">
+        <v>3</v>
+      </c>
+      <c r="G15" t="s">
+        <v>49</v>
+      </c>
+      <c r="H15" t="s">
+        <v>50</v>
+      </c>
+      <c r="J15" t="s">
+        <v>11</v>
+      </c>
+      <c r="K15" t="s">
+        <v>17</v>
+      </c>
+      <c r="L15" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="16" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B16" s="1">
+        <v>46321</v>
+      </c>
+      <c r="C16">
+        <v>10</v>
+      </c>
+      <c r="D16" s="6">
+        <v>0.33402777777777781</v>
+      </c>
+      <c r="E16" s="6">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="F16">
+        <v>2</v>
+      </c>
+      <c r="G16" t="s">
+        <v>52</v>
+      </c>
+      <c r="H16" t="s">
+        <v>53</v>
+      </c>
+      <c r="J16" t="s">
+        <v>54</v>
+      </c>
+      <c r="K16" t="s">
+        <v>17</v>
+      </c>
+      <c r="L16" t="s">
+        <v>55</v>
       </c>
     </row>
   </sheetData>
@@ -907,6 +1039,7 @@
     <hyperlink ref="I6" r:id="rId1"/>
     <hyperlink ref="I7" r:id="rId2"/>
     <hyperlink ref="I12" r:id="rId3"/>
+    <hyperlink ref="I13" r:id="rId4"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Upload day 14 tasks.
</commit_message>
<xml_diff>
--- a/timesheet/manoj_timesheet.xlsx
+++ b/timesheet/manoj_timesheet.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="57">
   <si>
     <t>Date</t>
   </si>
@@ -191,6 +191,9 @@
   </si>
   <si>
     <t>various functions used in pandas</t>
+  </si>
+  <si>
+    <t>https://github.com/manuhatescoding/mvj-internship-data-analytics/commit/f024863032a2d788a9d1c7b1fa825757df7ba641</t>
   </si>
 </sst>
 </file>
@@ -1024,6 +1027,9 @@
       <c r="H16" t="s">
         <v>53</v>
       </c>
+      <c r="I16" s="8" t="s">
+        <v>56</v>
+      </c>
       <c r="J16" t="s">
         <v>54</v>
       </c>
@@ -1040,6 +1046,7 @@
     <hyperlink ref="I7" r:id="rId2"/>
     <hyperlink ref="I12" r:id="rId3"/>
     <hyperlink ref="I13" r:id="rId4"/>
+    <hyperlink ref="I16" r:id="rId5"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>